<commit_message>
Checklist da fase de iniciação feito
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/BRA - Checklist Verificacao de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/BRA - Checklist Verificacao de Projeto.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D368FF4-D2F9-42B9-B2ED-71B733018A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0C6817-34FD-4E10-8215-AE31183EBF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
     <sheet name="Ver-Construção1" sheetId="3" r:id="rId5"/>
     <sheet name="Ver-Transição1" sheetId="4" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="119">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1052,6 +1052,21 @@
   </si>
   <si>
     <t>Foram realizados os testes de aceitação por parte do usuário final?</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Nunca foram atualizados</t>
+  </si>
+  <si>
+    <t>Fábio Adriano Silveira</t>
   </si>
 </sst>
 </file>
@@ -1384,7 +1399,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1453,7 +1468,13 @@
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1465,11 +1486,32 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1480,32 +1522,8 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1610,7 +1628,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.95238095238095233</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1845,10 +1863,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1866,10 +1884,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2095,7 +2113,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2181,22 +2199,22 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -7319,9 +7337,9 @@
       <c r="A3" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="20" t="e">
+      <c r="B3" s="20">
         <f>'Ver-Iniciação1'!$F$2</f>
-        <v>#DIV/0!</v>
+        <v>0.95238095238095233</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -7414,21 +7432,21 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="25" t="e">
+      <c r="B2" s="25">
         <f>('Ver-Iniciação1'!$G$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="C2" s="25">
         <f>('Ver-Iniciação1'!$H$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D2" s="25">
         <f>('Ver-Iniciação1'!$I$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E2" s="25">
         <f>('Ver-Iniciação1'!$J$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="N2" t="s">
         <v>2</v>
@@ -7454,21 +7472,21 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="25" t="e">
+      <c r="B3" s="25">
         <f>('Ver-Iniciação1'!$G$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C3" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="C3" s="25">
         <f>('Ver-Iniciação1'!$H$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D3" s="25">
         <f>('Ver-Iniciação1'!$I$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E3" s="25">
         <f>('Ver-Iniciação1'!$J$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="N3" t="s">
         <v>3</v>
@@ -7494,21 +7512,21 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="25" t="e">
+      <c r="B4" s="25">
         <f>('Ver-Iniciação1'!$G$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C4" s="25" t="e">
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="25">
         <f>('Ver-Iniciação1'!$H$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D4" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D4" s="25">
         <f>('Ver-Iniciação1'!$I$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E4" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E4" s="25">
         <f>('Ver-Iniciação1'!$J$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>#DIV/0!</v>
+        <v>0.2</v>
       </c>
       <c r="N4" t="s">
         <v>14</v>
@@ -7534,21 +7552,21 @@
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="25" t="e">
+      <c r="B5" s="25">
         <f>('Ver-Iniciação1'!$G$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="C5" s="25">
         <f>('Ver-Iniciação1'!$H$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D5" s="25">
         <f>('Ver-Iniciação1'!$I$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E5" s="25">
         <f>('Ver-Iniciação1'!$J$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="N5" t="s">
         <v>4</v>
@@ -7574,21 +7592,21 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="25" t="e">
+      <c r="B6" s="25">
         <f>('Ver-Iniciação1'!$G$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C6" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="C6" s="25">
         <f>('Ver-Iniciação1'!$H$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D6" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D6" s="25">
         <f>('Ver-Iniciação1'!$I$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E6" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E6" s="25">
         <f>('Ver-Iniciação1'!$J$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="N6" t="s">
         <v>36</v>
@@ -7614,21 +7632,21 @@
       <c r="A7" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="25" t="e">
+      <c r="B7" s="25">
         <f>('Ver-Iniciação1'!$G$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="C7" s="25">
         <f>('Ver-Iniciação1'!$H$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D7" s="25">
         <f>('Ver-Iniciação1'!$I$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E7" s="25">
         <f>('Ver-Iniciação1'!$J$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="N7" t="s">
         <v>5</v>
@@ -7734,21 +7752,21 @@
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="25" t="e">
+      <c r="B10" s="25">
         <f>('Ver-Iniciação1'!$G$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C10" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="C10" s="25">
         <f>('Ver-Iniciação1'!$H$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D10" s="25">
         <f>('Ver-Iniciação1'!$I$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="E10" s="25">
         <f>('Ver-Iniciação1'!$J$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="N10" t="s">
         <v>13</v>
@@ -7774,21 +7792,21 @@
       <c r="A11" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="25" t="e">
+      <c r="B11" s="25">
         <f>('Ver-Iniciação1'!$G$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C11" s="25" t="e">
+        <v>0.75</v>
+      </c>
+      <c r="C11" s="25">
         <f>('Ver-Iniciação1'!$H$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D11" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25">
         <f>('Ver-Iniciação1'!$I$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E11" s="25" t="e">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="25">
         <f>('Ver-Iniciação1'!$J$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="N11" t="s">
         <v>56</v>
@@ -8403,7 +8421,7 @@
   <cols>
     <col min="1" max="1" width="21.109375" customWidth="1"/>
     <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="84" style="2" customWidth="1"/>
+    <col min="3" max="3" width="89.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.88671875" customWidth="1"/>
     <col min="6" max="6" width="28" customWidth="1"/>
@@ -8414,41 +8432,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="32" t="s">
+      <c r="B2" s="33"/>
+      <c r="C2" s="28">
+        <v>46259</v>
+      </c>
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="33"/>
-      <c r="F2" s="21" t="e">
+      <c r="E2" s="40"/>
+      <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
-        <v>#DIV/0!</v>
+        <v>0.95238095238095233</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="42" t="s">
+      <c r="B3" s="33"/>
+      <c r="C3" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -8471,7 +8493,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="9"/>
@@ -8495,23 +8517,25 @@
       </c>
       <c r="J5">
         <f>COUNTIF(D6,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="40"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="9"/>
@@ -8523,7 +8547,7 @@
       <c r="F7" s="12"/>
       <c r="G7">
         <f>COUNTIF(D8:D12,"Sim")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H7">
         <f>COUNTIF(D8:D12,"Parcialmente")</f>
@@ -8539,67 +8563,77 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
-      <c r="A8" s="29"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="22">
         <v>2</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="29"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="29"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>4</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A11" s="29"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>5</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>6</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="29"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>3</v>
@@ -8609,7 +8643,7 @@
       <c r="F13" s="12"/>
       <c r="G13">
         <f>COUNTIF(D14:D18,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H13">
         <f>COUNTIF(D14:D18,"Parcialmente")</f>
@@ -8621,71 +8655,81 @@
       </c>
       <c r="J13">
         <f>COUNTIF(D14:D18,"NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="28.8">
-      <c r="A14" s="29"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="14.4">
+      <c r="A14" s="31"/>
       <c r="B14" s="23">
         <v>7</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A15" s="29"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="5">
         <v>8</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A16" s="29"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>9</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A17" s="29"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="23">
         <v>10</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A18" s="29"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="29"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="9"/>
       <c r="C19" s="10" t="s">
         <v>97</v>
@@ -8707,35 +8751,39 @@
       </c>
       <c r="J19">
         <f>COUNTIF(D20:D21,"NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="29"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="14.4">
+      <c r="A20" s="31"/>
       <c r="B20" s="23">
         <v>12</v>
       </c>
       <c r="C20" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="29"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="29"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="9"/>
       <c r="C22" s="10" t="s">
         <v>4</v>
@@ -8757,35 +8805,39 @@
       </c>
       <c r="J22">
         <f>COUNTIF(D23:D24,"NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="28.8">
-      <c r="A23" s="29"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="14.4">
+      <c r="A23" s="31"/>
       <c r="B23" s="23">
         <v>14</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="29"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="14.4">
-      <c r="A25" s="29"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="9"/>
       <c r="C25" s="10" t="s">
         <v>36</v>
@@ -8807,35 +8859,39 @@
       </c>
       <c r="J25">
         <f>COUNTIF(D26:D27,"NA")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="28.8">
-      <c r="A26" s="29"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="14.4">
+      <c r="A26" s="31"/>
       <c r="B26" s="23">
         <v>16</v>
       </c>
       <c r="C26" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="29"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>17</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="29"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>13</v>
@@ -8845,7 +8901,7 @@
       <c r="F28" s="12"/>
       <c r="G28">
         <f>COUNTIF(D29:D36,"Sim")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H28">
         <f>COUNTIF(D29:D36,"Parcialmente")</f>
@@ -8860,103 +8916,119 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.8">
-      <c r="A29" s="29"/>
+    <row r="29" spans="1:10" ht="14.4">
+      <c r="A29" s="31"/>
       <c r="B29" s="23">
         <v>21</v>
       </c>
       <c r="C29" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="29"/>
+      <c r="A30" s="31"/>
       <c r="B30" s="5">
         <v>22</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="29"/>
+      <c r="A31" s="31"/>
       <c r="B31" s="5">
         <v>23</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="29"/>
+      <c r="A32" s="31"/>
       <c r="B32" s="5">
         <v>24</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="29"/>
+      <c r="A33" s="31"/>
       <c r="B33" s="5">
         <v>25</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D33" s="3"/>
+      <c r="D33" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="29"/>
+      <c r="A34" s="31"/>
       <c r="B34" s="5">
         <v>26</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A35" s="29"/>
+      <c r="A35" s="31"/>
       <c r="B35" s="5">
         <v>27</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="3"/>
+      <c r="D35" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E35" s="8"/>
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="14.4">
-      <c r="A36" s="29"/>
+      <c r="A36" s="31"/>
       <c r="B36" s="5">
         <v>28</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="8"/>
+      <c r="D36" s="46" t="s">
+        <v>115</v>
+      </c>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1">
-      <c r="A37" s="38" t="s">
+      <c r="A37" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B37" s="9"/>
@@ -8968,7 +9040,7 @@
       <c r="F37" s="12"/>
       <c r="G37">
         <f>COUNTIF(D38:D41,"Sim")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H37">
         <f>COUNTIF(D38:D41,"Parcialmente")</f>
@@ -8976,59 +9048,69 @@
       </c>
       <c r="I37">
         <f>COUNTIF(D38:D41,"Não")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37">
         <f>COUNTIF(D38:D41,"NA")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="39"/>
+    <row r="38" spans="1:10" ht="14.4">
+      <c r="A38" s="30"/>
       <c r="B38" s="23">
         <v>30</v>
       </c>
       <c r="C38" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="39"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5">
         <v>31</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="39"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="20.25" customHeight="1">
-      <c r="A41" s="39"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D41" s="3"/>
-      <c r="E41" s="8"/>
+      <c r="D41" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>117</v>
+      </c>
       <c r="F41" s="8"/>
     </row>
   </sheetData>
@@ -9069,41 +9151,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="33"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D42)-COUNTIF(D5:D42,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="31"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9126,7 +9208,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9138,7 +9220,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="29"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9166,7 +9248,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="29"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9176,7 +9258,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="29"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9204,7 +9286,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A9" s="29"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -9220,7 +9302,7 @@
       <c r="J9"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="29"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10" t="s">
         <v>97</v>
@@ -9230,7 +9312,7 @@
       <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="29"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="23">
         <v>4</v>
       </c>
@@ -9258,7 +9340,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8">
-      <c r="A12" s="29"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="23">
         <v>5</v>
       </c>
@@ -9270,7 +9352,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="29"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="5">
         <v>6</v>
       </c>
@@ -9282,7 +9364,7 @@
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" ht="28.8">
-      <c r="A14" s="29"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>7</v>
       </c>
@@ -9294,7 +9376,7 @@
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" ht="14.4">
-      <c r="A15" s="29"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
         <v>4</v>
@@ -9304,7 +9386,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="29"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>7</v>
       </c>
@@ -9332,7 +9414,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="9"/>
@@ -9344,7 +9426,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="28.8">
-      <c r="A18" s="29"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -9372,7 +9454,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="29"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="23">
         <v>10</v>
       </c>
@@ -9384,7 +9466,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A20" s="29"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -9396,7 +9478,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="29"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>12</v>
       </c>
@@ -9408,7 +9490,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="9"/>
@@ -9420,7 +9502,7 @@
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="28.8">
-      <c r="A23" s="29"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="5">
         <v>17</v>
       </c>
@@ -9448,7 +9530,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="29"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>18</v>
       </c>
@@ -9460,7 +9542,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="29"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="5">
         <v>19</v>
       </c>
@@ -9472,7 +9554,7 @@
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="29"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="5">
         <v>21</v>
       </c>
@@ -9484,7 +9566,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="29"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>22</v>
       </c>
@@ -9496,7 +9578,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="9"/>
@@ -9508,7 +9590,7 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="37"/>
+      <c r="A29" s="42"/>
       <c r="B29" s="5">
         <v>23</v>
       </c>
@@ -9536,7 +9618,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="37"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -9548,7 +9630,7 @@
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="37"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>25</v>
       </c>
@@ -9560,7 +9642,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="37"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>26</v>
       </c>
@@ -9572,7 +9654,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="37"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>27</v>
       </c>
@@ -9584,7 +9666,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="37"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>28</v>
       </c>
@@ -9596,7 +9678,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="38" t="s">
+      <c r="A35" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -9608,7 +9690,7 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="39"/>
+      <c r="A36" s="30"/>
       <c r="B36" s="5">
         <v>29</v>
       </c>
@@ -9636,7 +9718,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="39"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>30</v>
       </c>
@@ -9648,7 +9730,7 @@
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="39"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>31</v>
       </c>
@@ -9660,7 +9742,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="39"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10" t="s">
         <v>15</v>
@@ -9670,7 +9752,7 @@
       <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="39"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
@@ -9698,7 +9780,7 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="39"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -9750,41 +9832,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="33"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D42,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="31"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9807,7 +9889,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9819,7 +9901,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="29"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9847,7 +9929,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="29"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9857,7 +9939,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="29"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9885,7 +9967,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="29"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>97</v>
@@ -9895,7 +9977,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="29"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -9923,7 +10005,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="29"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -9935,7 +10017,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -9947,7 +10029,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="29"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -9957,7 +10039,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="29"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -9985,7 +10067,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -9997,7 +10079,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="29"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10025,7 +10107,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.4">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10037,7 +10119,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="29"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -10065,7 +10147,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="29"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="5">
         <v>13</v>
       </c>
@@ -10077,7 +10159,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="29"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>14</v>
       </c>
@@ -10089,7 +10171,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="29"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>15</v>
       </c>
@@ -10101,7 +10183,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="29"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="5">
         <v>16</v>
       </c>
@@ -10113,7 +10195,7 @@
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="34" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="9"/>
@@ -10125,7 +10207,7 @@
       <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="29"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="23">
         <v>17</v>
       </c>
@@ -10153,7 +10235,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="29"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="5">
         <v>18</v>
       </c>
@@ -10165,7 +10247,7 @@
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="29"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="5">
         <v>19</v>
       </c>
@@ -10177,7 +10259,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="29"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>21</v>
       </c>
@@ -10189,7 +10271,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="29"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="5">
         <v>22</v>
       </c>
@@ -10201,7 +10283,7 @@
       <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B29" s="9"/>
@@ -10213,7 +10295,7 @@
       <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="37"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -10241,7 +10323,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="37"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>26</v>
       </c>
@@ -10253,7 +10335,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="37"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>27</v>
       </c>
@@ -10265,7 +10347,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="37"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>28</v>
       </c>
@@ -10277,7 +10359,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="37"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>29</v>
       </c>
@@ -10289,7 +10371,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="38" t="s">
+      <c r="A35" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -10301,7 +10383,7 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="39"/>
+      <c r="A36" s="30"/>
       <c r="B36" s="5">
         <v>30</v>
       </c>
@@ -10329,7 +10411,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="39"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>31</v>
       </c>
@@ -10341,7 +10423,7 @@
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="39"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>32</v>
       </c>
@@ -10353,7 +10435,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="39"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5"/>
       <c r="C39" s="8" t="s">
         <v>105</v>
@@ -10363,7 +10445,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="39"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="s">
         <v>15</v>
@@ -10373,7 +10455,7 @@
       <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="39"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -10401,7 +10483,7 @@
       </c>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="39"/>
+      <c r="A42" s="30"/>
       <c r="B42" s="5">
         <v>34</v>
       </c>
@@ -10482,41 +10564,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="31"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="33"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D43,"Sim")/(COUNTA(D5:D43)-COUNTIF(D5:D43,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="31"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="35"/>
-      <c r="F3" s="36"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -10539,7 +10621,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -10551,7 +10633,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="29"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -10579,7 +10661,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="29"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -10589,7 +10671,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="29"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -10617,7 +10699,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="29"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>14</v>
@@ -10627,7 +10709,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="29"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -10655,7 +10737,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="29"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10667,7 +10749,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A12" s="29"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10679,7 +10761,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="29"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10689,7 +10771,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="29"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10717,7 +10799,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10729,7 +10811,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="29"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10757,7 +10839,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10769,7 +10851,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="29"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -10797,7 +10879,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="29"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="5">
         <v>10</v>
       </c>
@@ -10809,7 +10891,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="29"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -10821,7 +10903,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="40"/>
+      <c r="A21" s="35"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -10833,7 +10915,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="34" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="9"/>
@@ -10845,7 +10927,7 @@
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="29"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="5">
         <v>14</v>
       </c>
@@ -10873,7 +10955,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="29"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -10885,7 +10967,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="34" t="s">
         <v>21</v>
       </c>
       <c r="B25" s="9"/>
@@ -10897,7 +10979,7 @@
       <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A26" s="29"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="23">
         <v>24</v>
       </c>
@@ -10925,7 +11007,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" s="1" customFormat="1" ht="43.2">
-      <c r="A27" s="29"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>25</v>
       </c>
@@ -10937,7 +11019,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="29"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>10</v>
@@ -10947,7 +11029,7 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="28.8">
-      <c r="A29" s="29"/>
+      <c r="A29" s="31"/>
       <c r="B29" s="23">
         <v>26</v>
       </c>
@@ -10975,7 +11057,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="9"/>
@@ -10987,7 +11069,7 @@
       <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="37"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>19</v>
       </c>
@@ -11015,7 +11097,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="28.8">
-      <c r="A32" s="37"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>20</v>
       </c>
@@ -11027,7 +11109,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="37"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>21</v>
       </c>
@@ -11039,7 +11121,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="37"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>24</v>
       </c>
@@ -11051,7 +11133,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="14.4">
-      <c r="A35" s="37"/>
+      <c r="A35" s="42"/>
       <c r="B35" s="5">
         <v>25</v>
       </c>
@@ -11063,7 +11145,7 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1">
-      <c r="A36" s="38" t="s">
+      <c r="A36" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B36" s="9"/>
@@ -11075,7 +11157,7 @@
       <c r="F36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="28.8">
-      <c r="A37" s="39"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>26</v>
       </c>
@@ -11103,7 +11185,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="14.4">
-      <c r="A38" s="39"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>27</v>
       </c>
@@ -11115,7 +11197,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="28.8">
-      <c r="A39" s="39"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5">
         <v>28</v>
       </c>
@@ -11127,7 +11209,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="39"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
         <v>105</v>
@@ -11137,7 +11219,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="39"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10" t="s">
         <v>15</v>
@@ -11147,7 +11229,7 @@
       <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="39"/>
+      <c r="A42" s="30"/>
       <c r="B42" s="5">
         <v>29</v>
       </c>
@@ -11175,7 +11257,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="14.4">
-      <c r="A43" s="39"/>
+      <c r="A43" s="30"/>
       <c r="B43" s="5">
         <v>30</v>
       </c>

</xml_diff>